<commit_message>
Fresh start - updated files
</commit_message>
<xml_diff>
--- a/region.xlsx
+++ b/region.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30219"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8BEEBA51-EAB5-4D45-AF31-01FF3C678D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7512A522-C5B3-4566-8276-D651604F2CA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
-    <t>Region Name</t>
+    <t>RegionName</t>
   </si>
   <si>
     <t>North-West</t>

</xml_diff>